<commit_message>
In-update ang mrf automation files
</commit_message>
<xml_diff>
--- a/PartsDatabase.xlsx
+++ b/PartsDatabase.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\N-20W1PF3VP3VC-Data\rabanes\Documents\mrf automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\My Apps\mrf automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3C1D3FC6-55DD-44DF-B856-C22D3FD0275C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE66810-0F98-460B-ACD7-2EB13CB6C40D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{DE375A06-EE60-4554-96B6-FF3DA3ED8F40}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DE375A06-EE60-4554-96B6-FF3DA3ED8F40}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="54">
   <si>
     <t>PART NUMBER</t>
   </si>
@@ -189,6 +189,18 @@
   </si>
   <si>
     <t>Plastic Cable Tie white</t>
+  </si>
+  <si>
+    <t>CATEGORY</t>
+  </si>
+  <si>
+    <t>EQUIPMENT</t>
+  </si>
+  <si>
+    <t>PERIPHERALS</t>
+  </si>
+  <si>
+    <t>MATERIALS</t>
   </si>
 </sst>
 </file>
@@ -270,7 +282,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -293,35 +305,16 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -336,6 +329,14 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -801,211 +802,287 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{356F8987-52F5-4415-A53D-8814C74CD30C}">
-  <dimension ref="A1:B25"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.6328125" customWidth="1"/>
-    <col min="2" max="2" width="52.90625" customWidth="1"/>
+    <col min="1" max="1" width="17.5703125" customWidth="1"/>
+    <col min="2" max="2" width="52.85546875" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="7" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="5" t="s">
+      <c r="C1" s="10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="7" t="s">
+      <c r="C2" s="8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="4" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
+      <c r="C3" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="7" t="s">
+      <c r="C4" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="7" t="s">
+      <c r="C5" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="7" t="s">
+      <c r="C6" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="7" t="s">
+      <c r="C7" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="4" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" s="5" t="s">
+      <c r="C8" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="4" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
+      <c r="C9" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
+      <c r="C10" s="8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A12" s="8" t="s">
+      <c r="C11" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="4" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
+      <c r="C12" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
+      <c r="C13" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
+      <c r="C14" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
+      <c r="C15" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" s="2" t="s">
+      <c r="C16" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="1" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" s="2" t="s">
+      <c r="C17" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" s="2" t="s">
+      <c r="C18" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" s="2" t="s">
+      <c r="C19" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="1" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" s="4" t="s">
+      <c r="C20" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="2" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" s="6" t="s">
+      <c r="C21" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="4" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" s="6" t="s">
+      <c r="C22" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="4" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A24" s="6" t="s">
+      <c r="C23" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="4" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A25" s="6" t="s">
+      <c r="C24" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="4" t="s">
         <v>49</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>